<commit_message>
Cập nhật tính năng xuất file excel dữ liêu Giảng viên
</commit_message>
<xml_diff>
--- a/demo_netcore_mvc/wwwroot/templates/SinhVienTheoGV_Template.xlsx
+++ b/demo_netcore_mvc/wwwroot/templates/SinhVienTheoGV_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\DOTNET\Repos\demo_netcore_mvc\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A999E8C-0235-4C30-8241-E8DFDD24370C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DADC0E00-B8E3-421E-AFF1-29E5149FFE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{13B07AF6-4011-4117-89DE-A39AD6BB70A5}"/>
   </bookViews>
@@ -36,27 +36,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Mã giảng viên: &lt;&lt;MaGV&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Họ tên: &lt;&lt;HoTenGV&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Khoa: &lt;&lt;TenKhoa&gt;&gt;</t>
-  </si>
-  <si>
-    <t>STT</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>MSSV</t>
   </si>
   <si>
-    <t>Họ tên</t>
-  </si>
-  <si>
-    <t>Khoa</t>
+    <t>Mã giảng viên</t>
+  </si>
+  <si>
+    <t>Họ tên giảng viên</t>
+  </si>
+  <si>
+    <t>Khoa gv</t>
+  </si>
+  <si>
+    <t>Lương</t>
+  </si>
+  <si>
+    <t>Họ tên sv</t>
+  </si>
+  <si>
+    <t>Khoa sv</t>
+  </si>
+  <si>
+    <t>Năm sinh</t>
+  </si>
+  <si>
+    <t>Quê quán</t>
+  </si>
+  <si>
+    <t>Đề tài</t>
   </si>
 </sst>
 </file>
@@ -428,36 +437,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29115306-A4C8-4ABD-9F98-DB68C60C3E0F}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
+      <c r="G1" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>